<commit_message>
Recalibrate prices to market sources (v1.2)
Freelance rates are now per project or per day, as Bogotá freelancers
quote, and anchored to published Colombian rate cards and price guides
for 2025–2026 (listed in doc 04, 2.6). Sale prices drop roughly by half
(pack 3 M, video de marca 4 M, clip 5.5 M, comercial 10 M, branding 4 M,
landing 2.5 M, sitio 7 M, retainer 3 M/mes), price floor to 2 M, margin
target to >= 50 %, cost-per-qualified-lead targets to 60–120 k.
Consequences propagated: full-time jump threshold raised to 30 M/month,
36-month scenarios re-run with market tickets and rule-based hiring,
launch tasks and ad copy updated. Spreadsheet and model scripts updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012v3e5faPpnQjnDf4ZwZMJ7
</commit_message>
<xml_diff>
--- a/docs/04-tabla-rentabilidad.xlsx
+++ b/docs/04-tabla-rentabilidad.xlsx
@@ -430,14 +430,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,79 +467,95 @@
           <t>Tarifa Rango (COP)</t>
         </is>
       </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Base / fuente</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DOP con equipo básico</t>
+          <t>DOP / videógrafo con equipo propio</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Jornada</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>800000</v>
+        <v>500000</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>1500000</v>
+        <v>900000</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>1000000</v>
+        <v>600000</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Alquiler FX3+lente 280–360k/día en Bogotá; operador 1,5–2,5× el alquiler</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DOP medio día</t>
+          <t>DOP media jornada</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Medio día</t>
+          <t>Media jornada</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>400000</v>
+        <v>300000</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>750000</v>
+        <v>500000</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>600000</v>
-      </c>
+        <v>350000</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Asistente de cámara</t>
+          <t>Asistente de cámara / gaffer</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Jornada</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E4" s="2" t="n">
         <v>200000</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E4" s="2" t="n">
-        <v>250000</v>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Salario junior 1,5–2 M/mes ÷ 10 jornadas</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gaffer</t>
+          <t>Sonidista con equipo</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Jornada</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -550,320 +567,466 @@
       <c r="E5" s="2" t="n">
         <v>300000</v>
       </c>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sonidista con equipo</t>
+          <t>Equipo extra (luces, gimbal, drone)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Jornada</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>350000</v>
+        <v>150000</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>600000</v>
+        <v>400000</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>450000</v>
+        <v>250000</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Casas de alquiler Bogotá</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Equipo extra (luces, gimbal, drone)</t>
+          <t>Edición reel / pieza corta</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Pieza</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>200000</v>
+        <v>80000</v>
       </c>
       <c r="D7" s="2" t="n">
-        <v>600000</v>
+        <v>250000</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>400000</v>
+        <v>100000</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>USD 20–60 por reel (LATAM)</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Editor/a de video</t>
+          <t>Edición pack 5 anuncios</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Hora</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>90000</v>
+        <v>400000</v>
       </c>
       <c r="D8" s="2" t="n">
-        <v>150000</v>
+        <v>700000</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>120000</v>
-      </c>
+        <v>500000</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Colorista</t>
+          <t>Edición clip musical / video de marca</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Pieza</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="D9" s="2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>700000</v>
       </c>
-      <c r="E9" s="2" t="n">
-        <v>500000</v>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Editor empleado 1,8–4 M/mes</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Motion graphics</t>
+          <t>Edición comercial 30s + cutdowns</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Pieza</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>400000</v>
+        <v>700000</v>
       </c>
       <c r="D10" s="2" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E10" s="2" t="n">
         <v>1000000</v>
       </c>
-      <c r="E10" s="2" t="n">
-        <v>600000</v>
-      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Diseñador/a de marca</t>
+          <t>Colorización</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Hora</t>
+          <t>Pieza</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>70000</v>
+        <v>200000</v>
       </c>
       <c r="D11" s="2" t="n">
-        <v>130000</v>
+        <v>500000</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>100000</v>
+        <v>300000</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Estimación; validar</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Diseño web no-code: landing</t>
+          <t>Animación de logo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Landing</t>
+          <t>Pieza</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>1000000</v>
+        <v>200000</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>1500000</v>
+        <v>500000</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>1200000</v>
+        <v>300000</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Marketplaces Colombia</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Diseño web no-code: sitio 5–7 pág.</t>
+          <t>Motion graphics 20–30 s</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sitio</t>
+          <t>Pieza</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>2500000</v>
+        <v>300000</v>
       </c>
       <c r="D13" s="2" t="n">
-        <v>4500000</v>
+        <v>800000</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>3500000</v>
+        <v>400000</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Estimación; validar</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Desarrollador/a a medida</t>
+          <t>Identidad de marca con manual (freelance)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Hora</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>120000</v>
+        <v>1200000</v>
       </c>
       <c r="D14" s="2" t="n">
-        <v>180000</v>
+        <v>2500000</v>
       </c>
       <c r="E14" s="2" t="n">
-        <v>150000</v>
+        <v>1500000</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Branding profesional Colombia 1,5–5,5 M</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Fotógrafo/a</t>
+          <t>Diseño de piezas para redes</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Sesión 3 h</t>
+          <t>Pieza</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>500000</v>
+        <v>30000</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>900000</v>
+        <v>80000</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>700000</v>
+        <v>50000</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Tarifarios diseño Colombia</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Copywriter</t>
+          <t>Web no-code: landing</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sitio</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>400000</v>
+        <v>600000</v>
       </c>
       <c r="D16" s="2" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="E16" s="2" t="n">
         <v>800000</v>
       </c>
-      <c r="E16" s="2" t="n">
-        <v>600000</v>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Landing Colombia 0,5–3 M</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Maquillaje y estilismo</t>
+          <t>Web no-code: sitio 5–7 páginas</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>200000</v>
+        <v>1500000</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>350000</v>
+        <v>3000000</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>280000</v>
+        <v>1800000</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Sitio corporativo Colombia 3–10 M</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Locación</t>
+          <t>Copywriting de sitio</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Proyecto</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>0</v>
+        <v>300000</v>
       </c>
       <c r="D18" s="2" t="n">
-        <v>800000</v>
+        <v>600000</v>
       </c>
       <c r="E18" s="2" t="n">
         <v>400000</v>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Estimación; validar</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Logística rodaje</t>
+          <t>Fotógrafo/a (sesión 2–3 h)</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Día</t>
+          <t>Sesión</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>250000</v>
+        <v>350000</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>500000</v>
+        <v>600000</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>350000</v>
+        <v>450000</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Retrato corporativo Bogotá desde 550k al público</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Maquillaje y estilismo</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Estimación; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Locación</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>400000</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Estimación; validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Logística rodaje</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Estimación</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Talento / modelo</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Día</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Jornada</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
         <v>300000</v>
       </c>
-      <c r="D20" s="2" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="E20" s="2" t="n">
+      <c r="D23" s="2" t="n">
         <v>800000</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>500000</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Estimación; validar</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -877,7 +1040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -957,14 +1120,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pack anuncios pauta (5 piezas, ½ día)</t>
+          <t>Pack 5 anuncios pauta (½ jornada)</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>6000000</v>
+        <v>3000000</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>2360000</v>
+        <v>1300000</v>
       </c>
       <c r="D4" s="2">
         <f>B4-C4</f>
@@ -975,7 +1138,7 @@
         <v/>
       </c>
       <c r="F4" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="G4" s="2">
         <f>F4*$B$1</f>
@@ -991,21 +1154,21 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>DOP ½ día 600k · editor 8h 960k · motion 600k · logística 200k</t>
+          <t>DOP ½ 350k · edición pack 500k · motion 300k · logística 150k</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Clip musical indie (1 día, equipo ligero)</t>
+          <t>Video de marca / corporativo 2–3 min</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10000000</v>
+        <v>4000000</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>4520000</v>
+        <v>2000000</v>
       </c>
       <c r="D5" s="2">
         <f>B5-C5</f>
@@ -1016,7 +1179,7 @@
         <v/>
       </c>
       <c r="F5" t="n">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="G5" s="2">
         <f>F5*$B$1</f>
@@ -1032,21 +1195,21 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>DOP 1M · asistente 250k · equipo 400k · editor 12h 1,44M · color 500k · locación 300k · maquillaje 280k · logística 350k</t>
+          <t>DOP 600k · sonido 300k · edición 700k · motion 200k · logística 200k</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Comercial marca mediana 30s + cutdowns</t>
+          <t>Clip musical indie (1 jornada)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>18000000</v>
+        <v>5500000</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>8090000</v>
+        <v>2650000</v>
       </c>
       <c r="D6" s="2">
         <f>B6-C6</f>
@@ -1057,7 +1220,7 @@
         <v/>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="G6" s="2">
         <f>F6*$B$1</f>
@@ -1073,21 +1236,21 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>DOP 1M · gaffer 300k · sonido 450k · equipo 600k · locación 800k · talento 800k · maquillaje 280k · editor 18h 2,16M · color 600k · motion 600k · logística 500k</t>
+          <t>DOP 600k · asistente 200k · equipo 250k · edición 700k · color 250k · locación 200k · maquillaje 200k · logística 250k</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Branding completo</t>
+          <t>Comercial 30s + 3 cutdowns (1 jornada)</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>8000000</v>
+        <v>10000000</v>
       </c>
       <c r="C7" s="2" t="n">
-        <v>3400000</v>
+        <v>4750000</v>
       </c>
       <c r="D7" s="2">
         <f>B7-C7</f>
@@ -1098,7 +1261,7 @@
         <v/>
       </c>
       <c r="F7" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G7" s="2">
         <f>F7*$B$1</f>
@@ -1114,21 +1277,21 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>diseño 25h 2,5M · motion logo 600k · mockups 300k</t>
+          <t>DOP 700k · gaffer 200k · sonido 350k · equipo 300k · locación 400k · talento 500k · maquillaje 200k · edición 1M · color 400k · motion 400k · logística 300k</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Landing + identidad express</t>
+          <t>Branding completo (freelance diseño)</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>4500000</v>
+        <v>4000000</v>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2000000</v>
+        <v>1900000</v>
       </c>
       <c r="D8" s="2">
         <f>B8-C8</f>
@@ -1139,7 +1302,7 @@
         <v/>
       </c>
       <c r="F8" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="G8" s="2">
         <f>F8*$B$1</f>
@@ -1155,21 +1318,21 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>web 1,2M · diseño 8h 800k</t>
+          <t>identidad + manual 1,5M · animación logo 300k · mockups 100k</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sitio corporativo 5–7 páginas</t>
+          <t>Landing + identidad express</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>13000000</v>
+        <v>2500000</v>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6300000</v>
+        <v>1200000</v>
       </c>
       <c r="D9" s="2">
         <f>B9-C9</f>
@@ -1180,7 +1343,7 @@
         <v/>
       </c>
       <c r="F9" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G9" s="2">
         <f>F9*$B$1</f>
@@ -1196,21 +1359,21 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>web 3,5M · diseño 15h 1,5M · copy 600k · fotos 700k</t>
+          <t>web 800k · diseño 400k</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Retainer Rango Lab (mensual)</t>
+          <t>Sitio corporativo 5–7 páginas</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>6000000</v>
+        <v>7000000</v>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2690000</v>
+        <v>3450000</v>
       </c>
       <c r="D10" s="2">
         <f>B10-C10</f>
@@ -1237,7 +1400,48 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>DOP ½ día 600k · editor 12h 1,44M · diseño 5h 500k · logística 150k</t>
+          <t>web 1,8M · diseño 800k · copy 400k · fotos 450k</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Retainer Rango Lab (mensual)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>1400000</v>
+      </c>
+      <c r="D11" s="2">
+        <f>B11-C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>D11/B11</f>
+        <v/>
+      </c>
+      <c r="F11" t="n">
+        <v>16</v>
+      </c>
+      <c r="G11" s="2">
+        <f>F11*$B$1</f>
+        <v/>
+      </c>
+      <c r="H11" s="2">
+        <f>D11-G11</f>
+        <v/>
+      </c>
+      <c r="I11" s="4">
+        <f>H11/B11</f>
+        <v/>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>DOP ½ 350k · edición 8 piezas 700k · diseño 250k · logística 100k</t>
         </is>
       </c>
     </row>
@@ -1252,14 +1456,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1270,22 +1476,32 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Fase 1 · 2 proy</t>
+          <t>F1 · 2 proy</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Fase 1 · 3 proy</t>
+          <t>F1 · 3 proy</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Fase 2a · 4 proy</t>
+          <t>F1 · 4 proy</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Fase 2b · 7 proy</t>
+          <t>F2a · 5 proy</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>F2a · 6 proy</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>F2b · 9 proy</t>
         </is>
       </c>
     </row>
@@ -1296,16 +1512,22 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>16000000</v>
+        <v>8500000</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>20500000</v>
+        <v>11000000</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>42000000</v>
+        <v>15000000</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>79000000</v>
+        <v>25500000</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>35500000</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>55500000</v>
       </c>
     </row>
     <row r="3">
@@ -1315,16 +1537,22 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>6880000</v>
+        <v>3950000</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>8880000</v>
+        <v>5150000</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>18700000</v>
+        <v>7150000</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>36340000</v>
+        <v>12000000</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>16850000</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>26450000</v>
       </c>
     </row>
     <row r="4">
@@ -1349,6 +1577,14 @@
         <f>E2-E3</f>
         <v/>
       </c>
+      <c r="F4" s="2">
+        <f>F2-F3</f>
+        <v/>
+      </c>
+      <c r="G4" s="2">
+        <f>G2-G3</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1357,15 +1593,21 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1100000</v>
+        <v>1000000</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1100000</v>
+        <v>1000000</v>
       </c>
       <c r="D5" s="2" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E5" s="2" t="n">
         <v>1800000</v>
       </c>
-      <c r="E5" s="2" t="n">
+      <c r="F5" s="2" t="n">
+        <v>1800000</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>3000000</v>
       </c>
     </row>
@@ -1376,15 +1618,21 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="D6" s="2" t="n">
+        <v>500000</v>
+      </c>
+      <c r="E6" s="2" t="n">
         <v>1200000</v>
       </c>
-      <c r="E6" s="2" t="n">
+      <c r="F6" s="2" t="n">
+        <v>1200000</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>1500000</v>
       </c>
     </row>
@@ -1401,9 +1649,15 @@
         <v>400000</v>
       </c>
       <c r="D7" s="2" t="n">
+        <v>400000</v>
+      </c>
+      <c r="E7" s="2" t="n">
         <v>500000</v>
       </c>
-      <c r="E7" s="2" t="n">
+      <c r="F7" s="2" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>600000</v>
       </c>
     </row>
@@ -1420,9 +1674,15 @@
         <v>0</v>
       </c>
       <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
         <v>900000</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="F8" s="2" t="n">
+        <v>900000</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>1800000</v>
       </c>
     </row>
@@ -1439,9 +1699,15 @@
         <v>300000</v>
       </c>
       <c r="D9" s="2" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E9" s="2" t="n">
         <v>500000</v>
       </c>
-      <c r="E9" s="2" t="n">
+      <c r="F9" s="2" t="n">
+        <v>500000</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>800000</v>
       </c>
     </row>
@@ -1467,6 +1733,14 @@
         <f>SUM(E5:E9)</f>
         <v/>
       </c>
+      <c r="F10" s="2">
+        <f>SUM(F5:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="2">
+        <f>SUM(G5:G9)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1481,9 +1755,15 @@
         <v>0</v>
       </c>
       <c r="D11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="2" t="n">
         <v>5200000</v>
       </c>
-      <c r="E11" s="2" t="n">
+      <c r="F11" s="2" t="n">
+        <v>5200000</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>11700000</v>
       </c>
     </row>
@@ -1500,9 +1780,15 @@
         <v>0.15</v>
       </c>
       <c r="D12" s="4" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E12" s="4" t="n">
         <v>0.05</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="F12" s="4" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1528,6 +1814,14 @@
         <f>E2*E12</f>
         <v/>
       </c>
+      <c r="F13" s="2">
+        <f>F2*F12</f>
+        <v/>
+      </c>
+      <c r="G13" s="2">
+        <f>G2*G12</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1551,6 +1845,14 @@
         <f>E4-E10-E11-E13</f>
         <v/>
       </c>
+      <c r="F14" s="2">
+        <f>F4-F10-F11-F13</f>
+        <v/>
+      </c>
+      <c r="G14" s="2">
+        <f>G4-G10-G11-G13</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1559,16 +1861,22 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C15" s="5" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="D15" s="5" t="n">
-        <v>135</v>
+        <v>74</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>245</v>
+        <v>122</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>162</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>238</v>
       </c>
     </row>
     <row r="16">
@@ -1584,9 +1892,15 @@
         <v>80</v>
       </c>
       <c r="D16" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="E16" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="F16" s="5" t="n">
+        <v>200</v>
+      </c>
+      <c r="G16" s="5" t="n">
         <v>320</v>
       </c>
     </row>

</xml_diff>